<commit_message>
Update campaign reports and reports-data.js for all 19 branches
</commit_message>
<xml_diff>
--- a/보고서/광주수완.xlsx
+++ b/보고서/광주수완.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="173">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="175">
   <si>
     <t>레뷰 캠페인 보고서</t>
   </si>
@@ -26,7 +26,7 @@
     <t>데이터 기준일자</t>
   </si>
   <si>
-    <t>2026-06-09</t>
+    <t>2026-06-14</t>
   </si>
   <si>
     <t xml:space="preserve">캠페인 정보 </t>
@@ -59,7 +59,7 @@
     <t xml:space="preserve">총 조회수 </t>
   </si>
   <si>
-    <t>126 (pv)</t>
+    <t>192 (pv)</t>
   </si>
   <si>
     <t xml:space="preserve">30일간 누적 조회수 </t>
@@ -68,7 +68,7 @@
     <t xml:space="preserve">일일 평균 조회수 </t>
   </si>
   <si>
-    <t>6 (pv)</t>
+    <t>7 (pv)</t>
   </si>
   <si>
     <t>유입 키워드 TOP 10</t>
@@ -81,6 +81,9 @@
   </si>
   <si>
     <t>비율(%)</t>
+  </si>
+  <si>
+    <t>광주독학재수학원</t>
   </si>
   <si>
     <t>광주 이투스 수완 주차</t>
@@ -167,7 +170,7 @@
     <t>일별 콘텐츠 조회수</t>
   </si>
   <si>
-    <t>날짜(2026.03.10~2026.06.09)</t>
+    <t>날짜(2026.03.15~2026.06.14)</t>
   </si>
   <si>
     <t>요일</t>
@@ -182,6 +185,36 @@
     <t>합산 조회수(PC+Mobile)</t>
   </si>
   <si>
+    <t>일</t>
+  </si>
+  <si>
+    <t>2026-06-13</t>
+  </si>
+  <si>
+    <t>토</t>
+  </si>
+  <si>
+    <t>2026-06-12</t>
+  </si>
+  <si>
+    <t>금</t>
+  </si>
+  <si>
+    <t>2026-06-11</t>
+  </si>
+  <si>
+    <t>목</t>
+  </si>
+  <si>
+    <t>2026-06-10</t>
+  </si>
+  <si>
+    <t>수</t>
+  </si>
+  <si>
+    <t>2026-06-09</t>
+  </si>
+  <si>
     <t>화</t>
   </si>
   <si>
@@ -194,31 +227,16 @@
     <t>2026-06-07</t>
   </si>
   <si>
-    <t>일</t>
-  </si>
-  <si>
     <t>2026-06-06</t>
-  </si>
-  <si>
-    <t>토</t>
   </si>
   <si>
     <t>2026-06-05</t>
   </si>
   <si>
-    <t>금</t>
-  </si>
-  <si>
     <t>2026-06-04</t>
   </si>
   <si>
-    <t>목</t>
-  </si>
-  <si>
     <t>2026-06-03</t>
-  </si>
-  <si>
-    <t>수</t>
   </si>
   <si>
     <t>2026-06-02</t>
@@ -461,21 +479,6 @@
     <t>2026-03-15</t>
   </si>
   <si>
-    <t>2026-03-14</t>
-  </si>
-  <si>
-    <t>2026-03-13</t>
-  </si>
-  <si>
-    <t>2026-03-12</t>
-  </si>
-  <si>
-    <t>2026-03-11</t>
-  </si>
-  <si>
-    <t>2026-03-10</t>
-  </si>
-  <si>
     <t>콘텐츠 목록</t>
   </si>
   <si>
@@ -537,6 +540,9 @@
   </si>
   <si>
     <t>이투스247학원 광주수완점</t>
+  </si>
+  <si>
+    <t>이투스247학원 후기</t>
   </si>
 </sst>
 </file>
@@ -1860,7 +1866,7 @@
       </c>
       <c r="E20" s="43"/>
       <c r="F20" s="43">
-        <v>0.5</v>
+        <v>0.33333333333333</v>
       </c>
       <c r="G20" s="24"/>
     </row>
@@ -1875,18 +1881,22 @@
       <c r="D21" s="27"/>
       <c r="E21" s="46"/>
       <c r="F21" s="46">
-        <v>0.5</v>
+        <v>0.33333333333333</v>
       </c>
       <c r="G21" s="24"/>
     </row>
     <row r="22" spans="1:26" customHeight="1" ht="15">
       <c r="A22" s="24"/>
       <c r="B22" s="41">
-        <v>3.0</v>
-      </c>
-      <c r="C22" s="15"/>
+        <v>3</v>
+      </c>
+      <c r="C22" s="15" t="s">
+        <v>23</v>
+      </c>
       <c r="E22" s="43"/>
-      <c r="F22" s="43"/>
+      <c r="F22" s="43">
+        <v>0.33333333333333</v>
+      </c>
       <c r="G22" s="24"/>
     </row>
     <row r="23" spans="1:26" customHeight="1" ht="15">
@@ -1975,7 +1985,7 @@
     <row r="31" spans="1:26" customHeight="1" ht="19.5">
       <c r="A31" s="24"/>
       <c r="B31" s="25" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C31" s="26"/>
       <c r="D31" s="26"/>
@@ -1986,34 +1996,34 @@
     <row r="32" spans="1:26" customHeight="1" ht="15">
       <c r="A32" s="3"/>
       <c r="B32" s="50" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C32" s="50" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D32" s="51" t="s">
         <v>20</v>
       </c>
       <c r="E32" s="40"/>
       <c r="F32" s="50" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G32" s="3"/>
     </row>
     <row r="33" spans="1:26" customHeight="1" ht="15">
       <c r="A33" s="52"/>
       <c r="B33" s="53" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C33" s="54" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D33" s="55">
         <v>0.90909090909091</v>
       </c>
       <c r="E33" s="27"/>
       <c r="F33" s="54" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G33" s="52"/>
     </row>
@@ -2021,30 +2031,30 @@
       <c r="A34" s="52"/>
       <c r="B34" s="56"/>
       <c r="C34" s="57" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D34" s="58">
         <v>0.090909090909091</v>
       </c>
       <c r="E34" s="59"/>
       <c r="F34" s="57" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G34" s="52"/>
     </row>
     <row r="35" spans="1:26" customHeight="1" ht="15">
       <c r="A35" s="52"/>
       <c r="B35" s="60" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C35" s="54" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D35" s="61">
         <v>0.68181818181818</v>
       </c>
       <c r="F35" s="54" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G35" s="52"/>
     </row>
@@ -2052,14 +2062,14 @@
       <c r="A36" s="52"/>
       <c r="B36" s="62"/>
       <c r="C36" s="44" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D36" s="63">
         <v>0.18181818181818</v>
       </c>
       <c r="E36" s="27"/>
       <c r="F36" s="44" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G36" s="52"/>
     </row>
@@ -2067,13 +2077,13 @@
       <c r="A37" s="52"/>
       <c r="B37" s="62"/>
       <c r="C37" s="54" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D37" s="61">
         <v>0.13636363636364</v>
       </c>
       <c r="F37" s="54" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G37" s="52"/>
     </row>
@@ -2089,16 +2099,16 @@
     <row r="39" spans="1:26" customHeight="1" ht="15">
       <c r="A39" s="52"/>
       <c r="B39" s="67" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C39" s="54" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D39" s="61">
         <v>0.8125</v>
       </c>
       <c r="F39" s="54" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G39" s="52"/>
     </row>
@@ -2106,14 +2116,14 @@
       <c r="A40" s="52"/>
       <c r="B40" s="62"/>
       <c r="C40" s="44" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D40" s="63">
         <v>0.125</v>
       </c>
       <c r="E40" s="27"/>
       <c r="F40" s="44" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G40" s="52"/>
     </row>
@@ -2121,13 +2131,13 @@
       <c r="A41" s="52"/>
       <c r="B41" s="62"/>
       <c r="C41" s="54" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D41" s="61">
         <v>0.0625</v>
       </c>
       <c r="F41" s="54" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G41" s="52"/>
     </row>
@@ -2143,17 +2153,17 @@
     <row r="43" spans="1:26" customHeight="1" ht="15">
       <c r="A43" s="52"/>
       <c r="B43" s="68" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C43" s="54" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D43" s="55">
         <v>1</v>
       </c>
       <c r="E43" s="27"/>
       <c r="F43" s="54" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G43" s="52"/>
       <c r="H43" s="69"/>
@@ -3284,7 +3294,7 @@
     <row r="1" spans="1:26" customHeight="1" ht="30">
       <c r="A1" s="74"/>
       <c r="B1" s="75" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C1" s="36"/>
       <c r="D1" s="36"/>
@@ -3295,20 +3305,20 @@
     <row r="2" spans="1:26" customHeight="1" ht="30">
       <c r="A2" s="76"/>
       <c r="B2" s="39" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C2" s="40"/>
       <c r="D2" s="77" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E2" s="77" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F2" s="78" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="G2" s="77" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="H2" s="69"/>
     </row>
@@ -3319,267 +3329,267 @@
       </c>
       <c r="C3"/>
       <c r="D3" s="81" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E3" s="82">
+        <v>4</v>
+      </c>
+      <c r="F3" s="82">
         <v>5</v>
       </c>
-      <c r="F3" s="82">
-        <v>2</v>
-      </c>
       <c r="G3" s="82">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="Z3" s="83"/>
     </row>
     <row r="4" spans="1:26" customHeight="1" ht="19.5">
       <c r="A4" s="79"/>
       <c r="B4" s="84" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C4" s="26"/>
       <c r="D4" s="85" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E4" s="86">
         <v>4</v>
       </c>
       <c r="F4" s="86">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="G4" s="86">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="Z4" s="83"/>
     </row>
     <row r="5" spans="1:26" customHeight="1" ht="19.5">
       <c r="A5" s="79"/>
       <c r="B5" s="80" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C5"/>
       <c r="D5" s="81" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E5" s="82">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F5" s="82">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="G5" s="82">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="Z5" s="83"/>
     </row>
     <row r="6" spans="1:26" customHeight="1" ht="19.5">
       <c r="A6" s="79"/>
       <c r="B6" s="84" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C6" s="26"/>
       <c r="D6" s="85" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E6" s="86">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="F6" s="86">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="G6" s="86">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="Z6" s="83"/>
     </row>
     <row r="7" spans="1:26" customHeight="1" ht="19.5">
       <c r="A7" s="79"/>
       <c r="B7" s="80" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C7"/>
       <c r="D7" s="81" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E7" s="82">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="F7" s="82">
         <v>5</v>
       </c>
       <c r="G7" s="82">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="Z7" s="83"/>
     </row>
     <row r="8" spans="1:26" customHeight="1" ht="19.5">
       <c r="A8" s="79"/>
       <c r="B8" s="84" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C8" s="26"/>
       <c r="D8" s="85" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E8" s="86">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="F8" s="86">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="G8" s="86">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="Z8" s="83"/>
     </row>
     <row r="9" spans="1:26" customHeight="1" ht="19.5">
       <c r="A9" s="79"/>
       <c r="B9" s="80" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C9"/>
       <c r="D9" s="81" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E9" s="82">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="F9" s="82">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="G9" s="82">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="Z9" s="83"/>
     </row>
     <row r="10" spans="1:26" customHeight="1" ht="19.5">
       <c r="A10" s="79"/>
       <c r="B10" s="84" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C10" s="26"/>
       <c r="D10" s="85" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E10" s="86">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="F10" s="86">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G10" s="86">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="Z10" s="83"/>
     </row>
     <row r="11" spans="1:26" customHeight="1" ht="19.5">
       <c r="A11" s="79"/>
       <c r="B11" s="80" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C11"/>
       <c r="D11" s="81" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E11" s="82">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F11" s="82">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G11" s="82">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="Z11" s="83"/>
     </row>
     <row r="12" spans="1:26" customHeight="1" ht="19.5">
       <c r="A12" s="79"/>
       <c r="B12" s="84" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C12" s="26"/>
       <c r="D12" s="85" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E12" s="86">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F12" s="86">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G12" s="86">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="Z12" s="83"/>
     </row>
     <row r="13" spans="1:26" customHeight="1" ht="19.5">
       <c r="A13" s="79"/>
       <c r="B13" s="80" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C13"/>
       <c r="D13" s="81" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E13" s="82">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="F13" s="82">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="G13" s="82">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="Z13" s="83"/>
     </row>
     <row r="14" spans="1:26" customHeight="1" ht="19.5">
       <c r="A14" s="79"/>
       <c r="B14" s="84" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C14" s="26"/>
       <c r="D14" s="85" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E14" s="86">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="F14" s="86">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="G14" s="86">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="Z14" s="83"/>
     </row>
     <row r="15" spans="1:26" customHeight="1" ht="19.5">
       <c r="A15" s="79"/>
       <c r="B15" s="80" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C15"/>
       <c r="D15" s="81" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E15" s="82">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="F15" s="82">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="G15" s="82">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="Z15" s="83"/>
     </row>
     <row r="16" spans="1:26" customHeight="1" ht="19.5">
       <c r="A16" s="79"/>
       <c r="B16" s="84" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C16" s="26"/>
       <c r="D16" s="85" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E16" s="86">
         <v>0</v>
@@ -3595,11 +3605,11 @@
     <row r="17" spans="1:26" customHeight="1" ht="19.5">
       <c r="A17" s="79"/>
       <c r="B17" s="80" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C17"/>
       <c r="D17" s="81" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E17" s="82">
         <v>0</v>
@@ -3615,11 +3625,11 @@
     <row r="18" spans="1:26" customHeight="1" ht="19.5">
       <c r="A18" s="79"/>
       <c r="B18" s="84" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C18" s="26"/>
       <c r="D18" s="85" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E18" s="86">
         <v>0</v>
@@ -3635,11 +3645,11 @@
     <row r="19" spans="1:26" customHeight="1" ht="19.5">
       <c r="A19" s="79"/>
       <c r="B19" s="80" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C19"/>
       <c r="D19" s="81" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E19" s="82">
         <v>0</v>
@@ -3655,11 +3665,11 @@
     <row r="20" spans="1:26" customHeight="1" ht="19.5">
       <c r="A20" s="79"/>
       <c r="B20" s="84" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C20" s="26"/>
       <c r="D20" s="85" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E20" s="86">
         <v>0</v>
@@ -3675,11 +3685,11 @@
     <row r="21" spans="1:26" customHeight="1" ht="19.5">
       <c r="A21" s="79"/>
       <c r="B21" s="80" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C21"/>
       <c r="D21" s="81" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E21" s="82">
         <v>0</v>
@@ -3695,11 +3705,11 @@
     <row r="22" spans="1:26" customHeight="1" ht="19.5">
       <c r="A22" s="79"/>
       <c r="B22" s="84" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C22" s="26"/>
       <c r="D22" s="85" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E22" s="86">
         <v>0</v>
@@ -3715,11 +3725,11 @@
     <row r="23" spans="1:26" customHeight="1" ht="19.5">
       <c r="A23" s="79"/>
       <c r="B23" s="80" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C23"/>
       <c r="D23" s="81" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E23" s="82">
         <v>0</v>
@@ -3735,11 +3745,11 @@
     <row r="24" spans="1:26" customHeight="1" ht="19.5">
       <c r="A24" s="79"/>
       <c r="B24" s="84" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C24" s="26"/>
       <c r="D24" s="85" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E24" s="86">
         <v>0</v>
@@ -3755,11 +3765,11 @@
     <row r="25" spans="1:26" customHeight="1" ht="19.5">
       <c r="A25" s="79"/>
       <c r="B25" s="80" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C25"/>
       <c r="D25" s="81" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E25" s="82">
         <v>0</v>
@@ -3775,11 +3785,11 @@
     <row r="26" spans="1:26" customHeight="1" ht="19.5">
       <c r="A26" s="79"/>
       <c r="B26" s="84" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C26" s="26"/>
       <c r="D26" s="85" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E26" s="86">
         <v>0</v>
@@ -3795,11 +3805,11 @@
     <row r="27" spans="1:26" customHeight="1" ht="19.5">
       <c r="A27" s="79"/>
       <c r="B27" s="80" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C27"/>
       <c r="D27" s="81" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E27" s="82">
         <v>0</v>
@@ -3815,11 +3825,11 @@
     <row r="28" spans="1:26" customHeight="1" ht="19.5">
       <c r="A28" s="79"/>
       <c r="B28" s="84" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C28" s="26"/>
       <c r="D28" s="85" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E28" s="86">
         <v>0</v>
@@ -3835,11 +3845,11 @@
     <row r="29" spans="1:26" customHeight="1" ht="19.5">
       <c r="A29" s="79"/>
       <c r="B29" s="80" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C29"/>
       <c r="D29" s="81" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E29" s="82">
         <v>0</v>
@@ -3855,11 +3865,11 @@
     <row r="30" spans="1:26" customHeight="1" ht="19.5">
       <c r="A30" s="79"/>
       <c r="B30" s="84" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C30" s="26"/>
       <c r="D30" s="85" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E30" s="86">
         <v>0</v>
@@ -3875,11 +3885,11 @@
     <row r="31" spans="1:26" customHeight="1" ht="19.5">
       <c r="A31" s="79"/>
       <c r="B31" s="80" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C31"/>
       <c r="D31" s="81" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E31" s="82">
         <v>0</v>
@@ -3895,11 +3905,11 @@
     <row r="32" spans="1:26" customHeight="1" ht="19.5">
       <c r="A32" s="79"/>
       <c r="B32" s="84" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C32" s="26"/>
       <c r="D32" s="85" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E32" s="86">
         <v>0</v>
@@ -3915,11 +3925,11 @@
     <row r="33" spans="1:26" customHeight="1" ht="19.5">
       <c r="A33" s="79"/>
       <c r="B33" s="80" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C33"/>
       <c r="D33" s="81" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E33" s="82">
         <v>0</v>
@@ -3935,11 +3945,11 @@
     <row r="34" spans="1:26" customHeight="1" ht="19.5">
       <c r="A34" s="79"/>
       <c r="B34" s="84" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C34" s="26"/>
       <c r="D34" s="85" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E34" s="86">
         <v>0</v>
@@ -3955,11 +3965,11 @@
     <row r="35" spans="1:26" customHeight="1" ht="19.5">
       <c r="A35" s="79"/>
       <c r="B35" s="80" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C35"/>
       <c r="D35" s="81" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E35" s="82">
         <v>0</v>
@@ -3975,11 +3985,11 @@
     <row r="36" spans="1:26" customHeight="1" ht="19.5">
       <c r="A36" s="79"/>
       <c r="B36" s="84" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C36" s="26"/>
       <c r="D36" s="85" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E36" s="86">
         <v>0</v>
@@ -3995,11 +4005,11 @@
     <row r="37" spans="1:26" customHeight="1" ht="19.5">
       <c r="A37" s="79"/>
       <c r="B37" s="80" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C37"/>
       <c r="D37" s="81" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E37" s="82">
         <v>0</v>
@@ -4015,11 +4025,11 @@
     <row r="38" spans="1:26" customHeight="1" ht="19.5">
       <c r="A38" s="79"/>
       <c r="B38" s="84" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C38" s="26"/>
       <c r="D38" s="85" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E38" s="86">
         <v>0</v>
@@ -4035,11 +4045,11 @@
     <row r="39" spans="1:26" customHeight="1" ht="19.5">
       <c r="A39" s="79"/>
       <c r="B39" s="80" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C39"/>
       <c r="D39" s="81" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E39" s="82">
         <v>0</v>
@@ -4055,11 +4065,11 @@
     <row r="40" spans="1:26" customHeight="1" ht="19.5">
       <c r="A40" s="79"/>
       <c r="B40" s="84" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C40" s="26"/>
       <c r="D40" s="85" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E40" s="86">
         <v>0</v>
@@ -4075,11 +4085,11 @@
     <row r="41" spans="1:26" customHeight="1" ht="19.5">
       <c r="A41" s="79"/>
       <c r="B41" s="80" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C41"/>
       <c r="D41" s="81" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E41" s="82">
         <v>0</v>
@@ -4095,11 +4105,11 @@
     <row r="42" spans="1:26" customHeight="1" ht="19.5">
       <c r="A42" s="79"/>
       <c r="B42" s="84" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C42" s="26"/>
       <c r="D42" s="85" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E42" s="86">
         <v>0</v>
@@ -4115,11 +4125,11 @@
     <row r="43" spans="1:26" customHeight="1" ht="19.5">
       <c r="A43" s="79"/>
       <c r="B43" s="80" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C43"/>
       <c r="D43" s="81" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E43" s="82">
         <v>0</v>
@@ -4135,11 +4145,11 @@
     <row r="44" spans="1:26" customHeight="1" ht="19.5">
       <c r="A44" s="79"/>
       <c r="B44" s="84" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C44" s="26"/>
       <c r="D44" s="85" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E44" s="86">
         <v>0</v>
@@ -4155,11 +4165,11 @@
     <row r="45" spans="1:26" customHeight="1" ht="19.5">
       <c r="A45" s="79"/>
       <c r="B45" s="80" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C45"/>
       <c r="D45" s="81" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E45" s="82">
         <v>0</v>
@@ -4175,11 +4185,11 @@
     <row r="46" spans="1:26" customHeight="1" ht="19.5">
       <c r="A46" s="79"/>
       <c r="B46" s="84" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C46" s="26"/>
       <c r="D46" s="85" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E46" s="86">
         <v>0</v>
@@ -4195,11 +4205,11 @@
     <row r="47" spans="1:26" customHeight="1" ht="19.5">
       <c r="A47" s="79"/>
       <c r="B47" s="80" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C47"/>
       <c r="D47" s="81" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E47" s="82">
         <v>0</v>
@@ -4215,11 +4225,11 @@
     <row r="48" spans="1:26" customHeight="1" ht="19.5">
       <c r="A48" s="79"/>
       <c r="B48" s="84" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C48" s="26"/>
       <c r="D48" s="85" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E48" s="86">
         <v>0</v>
@@ -4235,11 +4245,11 @@
     <row r="49" spans="1:26" customHeight="1" ht="19.5">
       <c r="A49" s="79"/>
       <c r="B49" s="80" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C49"/>
       <c r="D49" s="81" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E49" s="82">
         <v>0</v>
@@ -4255,11 +4265,11 @@
     <row r="50" spans="1:26" customHeight="1" ht="19.5">
       <c r="A50" s="79"/>
       <c r="B50" s="84" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C50" s="26"/>
       <c r="D50" s="85" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E50" s="86">
         <v>0</v>
@@ -4275,11 +4285,11 @@
     <row r="51" spans="1:26" customHeight="1" ht="19.5">
       <c r="A51" s="79"/>
       <c r="B51" s="80" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C51"/>
       <c r="D51" s="81" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E51" s="82">
         <v>0</v>
@@ -4295,11 +4305,11 @@
     <row r="52" spans="1:26" customHeight="1" ht="19.5">
       <c r="A52" s="79"/>
       <c r="B52" s="84" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C52" s="26"/>
       <c r="D52" s="85" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E52" s="86">
         <v>0</v>
@@ -4315,11 +4325,11 @@
     <row r="53" spans="1:26" customHeight="1" ht="19.5">
       <c r="A53" s="79"/>
       <c r="B53" s="80" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C53"/>
       <c r="D53" s="81" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E53" s="82">
         <v>0</v>
@@ -4335,11 +4345,11 @@
     <row r="54" spans="1:26" customHeight="1" ht="19.5">
       <c r="A54" s="79"/>
       <c r="B54" s="84" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C54" s="26"/>
       <c r="D54" s="85" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E54" s="86">
         <v>0</v>
@@ -4355,11 +4365,11 @@
     <row r="55" spans="1:26" customHeight="1" ht="19.5">
       <c r="A55" s="79"/>
       <c r="B55" s="80" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C55"/>
       <c r="D55" s="81" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E55" s="82">
         <v>0</v>
@@ -4375,11 +4385,11 @@
     <row r="56" spans="1:26" customHeight="1" ht="19.5">
       <c r="A56" s="79"/>
       <c r="B56" s="84" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C56" s="26"/>
       <c r="D56" s="85" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E56" s="86">
         <v>0</v>
@@ -4395,11 +4405,11 @@
     <row r="57" spans="1:26" customHeight="1" ht="19.5">
       <c r="A57" s="79"/>
       <c r="B57" s="80" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C57"/>
       <c r="D57" s="81" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E57" s="82">
         <v>0</v>
@@ -4415,11 +4425,11 @@
     <row r="58" spans="1:26" customHeight="1" ht="19.5">
       <c r="A58" s="79"/>
       <c r="B58" s="84" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C58" s="26"/>
       <c r="D58" s="85" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E58" s="86">
         <v>0</v>
@@ -4435,11 +4445,11 @@
     <row r="59" spans="1:26" customHeight="1" ht="19.5">
       <c r="A59" s="79"/>
       <c r="B59" s="80" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C59"/>
       <c r="D59" s="81" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E59" s="82">
         <v>0</v>
@@ -4455,11 +4465,11 @@
     <row r="60" spans="1:26" customHeight="1" ht="19.5">
       <c r="A60" s="79"/>
       <c r="B60" s="84" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C60" s="26"/>
       <c r="D60" s="85" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E60" s="86">
         <v>0</v>
@@ -4475,11 +4485,11 @@
     <row r="61" spans="1:26" customHeight="1" ht="19.5">
       <c r="A61" s="79"/>
       <c r="B61" s="80" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C61"/>
       <c r="D61" s="81" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E61" s="82">
         <v>0</v>
@@ -4495,11 +4505,11 @@
     <row r="62" spans="1:26" customHeight="1" ht="19.5">
       <c r="A62" s="79"/>
       <c r="B62" s="84" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C62" s="26"/>
       <c r="D62" s="85" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E62" s="86">
         <v>0</v>
@@ -4515,11 +4525,11 @@
     <row r="63" spans="1:26" customHeight="1" ht="19.5">
       <c r="A63" s="79"/>
       <c r="B63" s="80" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C63"/>
       <c r="D63" s="81" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E63" s="82">
         <v>0</v>
@@ -4535,11 +4545,11 @@
     <row r="64" spans="1:26" customHeight="1" ht="19.5">
       <c r="A64" s="79"/>
       <c r="B64" s="84" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C64" s="26"/>
       <c r="D64" s="85" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E64" s="86">
         <v>0</v>
@@ -4555,11 +4565,11 @@
     <row r="65" spans="1:26" customHeight="1" ht="19.5">
       <c r="A65" s="79"/>
       <c r="B65" s="80" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C65"/>
       <c r="D65" s="81" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E65" s="82">
         <v>0</v>
@@ -4575,11 +4585,11 @@
     <row r="66" spans="1:26" customHeight="1" ht="19.5">
       <c r="A66" s="79"/>
       <c r="B66" s="84" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C66" s="26"/>
       <c r="D66" s="85" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E66" s="86">
         <v>0</v>
@@ -4595,11 +4605,11 @@
     <row r="67" spans="1:26" customHeight="1" ht="19.5">
       <c r="A67" s="79"/>
       <c r="B67" s="80" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C67"/>
       <c r="D67" s="81" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E67" s="82">
         <v>0</v>
@@ -4615,11 +4625,11 @@
     <row r="68" spans="1:26" customHeight="1" ht="19.5">
       <c r="A68" s="79"/>
       <c r="B68" s="84" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C68" s="26"/>
       <c r="D68" s="85" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E68" s="86">
         <v>0</v>
@@ -4635,11 +4645,11 @@
     <row r="69" spans="1:26" customHeight="1" ht="19.5">
       <c r="A69" s="79"/>
       <c r="B69" s="80" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C69"/>
       <c r="D69" s="81" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E69" s="82">
         <v>0</v>
@@ -4655,11 +4665,11 @@
     <row r="70" spans="1:26" customHeight="1" ht="19.5">
       <c r="A70" s="79"/>
       <c r="B70" s="84" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C70" s="26"/>
       <c r="D70" s="85" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E70" s="86">
         <v>0</v>
@@ -4675,11 +4685,11 @@
     <row r="71" spans="1:26" customHeight="1" ht="19.5">
       <c r="A71" s="79"/>
       <c r="B71" s="80" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C71"/>
       <c r="D71" s="81" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E71" s="82">
         <v>0</v>
@@ -4695,11 +4705,11 @@
     <row r="72" spans="1:26" customHeight="1" ht="19.5">
       <c r="A72" s="79"/>
       <c r="B72" s="84" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C72" s="26"/>
       <c r="D72" s="85" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E72" s="86">
         <v>0</v>
@@ -4715,11 +4725,11 @@
     <row r="73" spans="1:26" customHeight="1" ht="19.5">
       <c r="A73" s="79"/>
       <c r="B73" s="80" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C73"/>
       <c r="D73" s="81" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E73" s="82">
         <v>0</v>
@@ -4735,11 +4745,11 @@
     <row r="74" spans="1:26" customHeight="1" ht="19.5">
       <c r="A74" s="79"/>
       <c r="B74" s="84" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C74" s="26"/>
       <c r="D74" s="85" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E74" s="86">
         <v>0</v>
@@ -4755,11 +4765,11 @@
     <row r="75" spans="1:26" customHeight="1" ht="19.5">
       <c r="A75" s="79"/>
       <c r="B75" s="80" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C75"/>
       <c r="D75" s="81" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E75" s="82">
         <v>0</v>
@@ -4775,11 +4785,11 @@
     <row r="76" spans="1:26" customHeight="1" ht="19.5">
       <c r="A76" s="79"/>
       <c r="B76" s="84" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C76" s="26"/>
       <c r="D76" s="85" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E76" s="86">
         <v>0</v>
@@ -4795,11 +4805,11 @@
     <row r="77" spans="1:26" customHeight="1" ht="19.5">
       <c r="A77" s="79"/>
       <c r="B77" s="80" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C77"/>
       <c r="D77" s="81" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E77" s="82">
         <v>0</v>
@@ -4815,11 +4825,11 @@
     <row r="78" spans="1:26" customHeight="1" ht="19.5">
       <c r="A78" s="79"/>
       <c r="B78" s="84" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C78" s="26"/>
       <c r="D78" s="85" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E78" s="86">
         <v>0</v>
@@ -4835,11 +4845,11 @@
     <row r="79" spans="1:26" customHeight="1" ht="19.5">
       <c r="A79" s="79"/>
       <c r="B79" s="80" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C79"/>
       <c r="D79" s="81" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E79" s="82">
         <v>0</v>
@@ -4855,11 +4865,11 @@
     <row r="80" spans="1:26" customHeight="1" ht="19.5">
       <c r="A80" s="79"/>
       <c r="B80" s="84" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C80" s="26"/>
       <c r="D80" s="85" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E80" s="86">
         <v>0</v>
@@ -4875,11 +4885,11 @@
     <row r="81" spans="1:26" customHeight="1" ht="19.5">
       <c r="A81" s="79"/>
       <c r="B81" s="80" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C81"/>
       <c r="D81" s="81" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E81" s="82">
         <v>0</v>
@@ -4895,11 +4905,11 @@
     <row r="82" spans="1:26" customHeight="1" ht="19.5">
       <c r="A82" s="79"/>
       <c r="B82" s="84" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C82" s="26"/>
       <c r="D82" s="85" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E82" s="86">
         <v>0</v>
@@ -4915,11 +4925,11 @@
     <row r="83" spans="1:26" customHeight="1" ht="19.5">
       <c r="A83" s="79"/>
       <c r="B83" s="80" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C83"/>
       <c r="D83" s="81" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E83" s="82">
         <v>0</v>
@@ -4935,11 +4945,11 @@
     <row r="84" spans="1:26" customHeight="1" ht="19.5">
       <c r="A84" s="79"/>
       <c r="B84" s="84" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C84" s="26"/>
       <c r="D84" s="85" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E84" s="86">
         <v>0</v>
@@ -4955,11 +4965,11 @@
     <row r="85" spans="1:26" customHeight="1" ht="19.5">
       <c r="A85" s="79"/>
       <c r="B85" s="80" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C85"/>
       <c r="D85" s="81" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E85" s="82">
         <v>0</v>
@@ -4975,11 +4985,11 @@
     <row r="86" spans="1:26" customHeight="1" ht="19.5">
       <c r="A86" s="79"/>
       <c r="B86" s="84" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C86" s="26"/>
       <c r="D86" s="85" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E86" s="86">
         <v>0</v>
@@ -4995,11 +5005,11 @@
     <row r="87" spans="1:26" customHeight="1" ht="19.5">
       <c r="A87" s="79"/>
       <c r="B87" s="80" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C87"/>
       <c r="D87" s="81" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E87" s="82">
         <v>0</v>
@@ -5015,11 +5025,11 @@
     <row r="88" spans="1:26" customHeight="1" ht="19.5">
       <c r="A88" s="79"/>
       <c r="B88" s="84" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C88" s="26"/>
       <c r="D88" s="85" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E88" s="86">
         <v>0</v>
@@ -5035,11 +5045,11 @@
     <row r="89" spans="1:26" customHeight="1" ht="19.5">
       <c r="A89" s="79"/>
       <c r="B89" s="80" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C89"/>
       <c r="D89" s="81" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E89" s="82">
         <v>0</v>
@@ -5055,11 +5065,11 @@
     <row r="90" spans="1:26" customHeight="1" ht="19.5">
       <c r="A90" s="79"/>
       <c r="B90" s="84" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C90" s="26"/>
       <c r="D90" s="85" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E90" s="86">
         <v>0</v>
@@ -5075,11 +5085,11 @@
     <row r="91" spans="1:26" customHeight="1" ht="19.5">
       <c r="A91" s="79"/>
       <c r="B91" s="80" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C91"/>
       <c r="D91" s="81" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E91" s="82">
         <v>0</v>
@@ -5095,11 +5105,11 @@
     <row r="92" spans="1:26" customHeight="1" ht="19.5">
       <c r="A92" s="79"/>
       <c r="B92" s="84" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C92" s="26"/>
       <c r="D92" s="85" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E92" s="86">
         <v>0</v>
@@ -5115,11 +5125,11 @@
     <row r="93" spans="1:26" customHeight="1" ht="19.5">
       <c r="A93" s="79"/>
       <c r="B93" s="80" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C93"/>
       <c r="D93" s="81" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E93" s="82">
         <v>0</v>
@@ -5135,11 +5145,11 @@
     <row r="94" spans="1:26" customHeight="1" ht="19.5">
       <c r="A94" s="79"/>
       <c r="B94" s="84" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C94" s="26"/>
       <c r="D94" s="85" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E94" s="86">
         <v>0</v>
@@ -13432,7 +13442,7 @@
     <row r="1" spans="1:26" customHeight="1" ht="30">
       <c r="A1" s="89"/>
       <c r="B1" s="90" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C1" s="26"/>
       <c r="D1" s="26"/>
@@ -13444,19 +13454,19 @@
     <row r="2" spans="1:26" customHeight="1" ht="24.75">
       <c r="A2" s="83"/>
       <c r="B2" s="91" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C2" s="92" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D2" s="91" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="E2" s="91" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="F2" s="91" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="G2" s="83"/>
       <c r="H2" s="89"/>
@@ -13464,13 +13474,13 @@
     <row r="3" spans="1:26" customHeight="1" ht="27.75">
       <c r="A3" s="89"/>
       <c r="B3" s="93" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C3" s="24" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D3" s="94" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="E3" s="24">
         <v>3</v>
@@ -13485,7 +13495,7 @@
     <row r="4" spans="1:26" customHeight="1" ht="15">
       <c r="A4" s="89"/>
       <c r="B4" s="96" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C4"/>
       <c r="D4"/>
@@ -13498,13 +13508,13 @@
     <row r="5" spans="1:26" customHeight="1" ht="27.75">
       <c r="A5" s="89"/>
       <c r="B5" s="97" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C5" s="98" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D5" s="99" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="E5" s="98">
         <v>6</v>
@@ -13519,7 +13529,7 @@
     <row r="6" spans="1:26" customHeight="1" ht="15">
       <c r="A6" s="95"/>
       <c r="B6" s="100" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C6" s="26"/>
       <c r="D6" s="26"/>
@@ -13532,13 +13542,13 @@
     <row r="7" spans="1:26" customHeight="1" ht="27.75">
       <c r="A7" s="89"/>
       <c r="B7" s="93" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C7" s="24" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D7" s="94" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="E7" s="24">
         <v>3</v>
@@ -13553,7 +13563,7 @@
     <row r="8" spans="1:26" customHeight="1" ht="15">
       <c r="A8" s="89"/>
       <c r="B8" s="96" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C8"/>
       <c r="D8"/>
@@ -13566,7 +13576,7 @@
     <row r="9" spans="1:26" customHeight="1" ht="24">
       <c r="A9" s="89"/>
       <c r="B9" s="101" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C9" s="26"/>
       <c r="D9" s="27"/>
@@ -23495,7 +23505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Z1000"/>
+  <dimension ref="A1:Z1001"/>
   <sheetFormatPr customHeight="true" defaultRowHeight="15" defaultColWidth="14.43" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="18.86" customWidth="true" style="0"/>
@@ -23525,7 +23535,7 @@
   <sheetData>
     <row r="1" spans="1:26" customHeight="1" ht="30">
       <c r="A1" s="103" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="2" spans="1:26" customHeight="1" ht="18">
@@ -23533,7 +23543,7 @@
         <v>19</v>
       </c>
       <c r="B2" s="105" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C2" s="106"/>
       <c r="D2" s="106"/>
@@ -23556,7 +23566,7 @@
       <c r="U2" s="106"/>
       <c r="V2" s="107"/>
       <c r="W2" s="108" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="3" spans="1:26" customHeight="1" ht="24.75">
@@ -23628,7 +23638,7 @@
     </row>
     <row r="4" spans="1:26" customHeight="1" ht="18">
       <c r="A4" s="112" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B4" s="113">
         <v>0</v>
@@ -23701,7 +23711,7 @@
     </row>
     <row r="5" spans="1:26" customHeight="1" ht="18">
       <c r="A5" s="114" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B5" s="115">
         <v>0</v>
@@ -23772,30 +23782,78 @@
       </c>
       <c r="Z5"/>
     </row>
-    <row r="6" spans="1:26" customHeight="1" ht="15.75">
-      <c r="A6" s="116"/>
-      <c r="B6" s="116"/>
-      <c r="C6" s="116"/>
-      <c r="D6" s="116"/>
-      <c r="E6" s="116"/>
-      <c r="F6" s="116"/>
-      <c r="G6" s="116"/>
-      <c r="H6" s="116"/>
-      <c r="I6" s="116"/>
-      <c r="J6" s="116"/>
-      <c r="K6" s="116"/>
-      <c r="L6" s="116"/>
-      <c r="M6" s="116"/>
-      <c r="N6" s="116"/>
-      <c r="O6" s="116"/>
-      <c r="P6" s="116"/>
-      <c r="Q6" s="116"/>
-      <c r="R6" s="116"/>
-      <c r="S6" s="116"/>
-      <c r="T6" s="116"/>
-      <c r="U6" s="116"/>
-      <c r="V6" s="116"/>
-      <c r="W6" s="116"/>
+    <row r="6" spans="1:26" customHeight="1" ht="18">
+      <c r="A6" s="112" t="s">
+        <v>174</v>
+      </c>
+      <c r="B6" s="113">
+        <v>0</v>
+      </c>
+      <c r="C6" s="113">
+        <v>0</v>
+      </c>
+      <c r="D6" s="113">
+        <v>0</v>
+      </c>
+      <c r="E6" s="113">
+        <v>0</v>
+      </c>
+      <c r="F6" s="113">
+        <v>0</v>
+      </c>
+      <c r="G6" s="113">
+        <v>0</v>
+      </c>
+      <c r="H6" s="113">
+        <v>0</v>
+      </c>
+      <c r="I6" s="113">
+        <v>0</v>
+      </c>
+      <c r="J6" s="113">
+        <v>0</v>
+      </c>
+      <c r="K6" s="113">
+        <v>0</v>
+      </c>
+      <c r="L6" s="113">
+        <v>0</v>
+      </c>
+      <c r="M6" s="113">
+        <v>0</v>
+      </c>
+      <c r="N6" s="113">
+        <v>0</v>
+      </c>
+      <c r="O6" s="113">
+        <v>0</v>
+      </c>
+      <c r="P6" s="113">
+        <v>0</v>
+      </c>
+      <c r="Q6" s="113">
+        <v>0</v>
+      </c>
+      <c r="R6" s="113">
+        <v>0</v>
+      </c>
+      <c r="S6" s="113">
+        <v>0</v>
+      </c>
+      <c r="T6" s="113">
+        <v>0</v>
+      </c>
+      <c r="U6" s="113">
+        <v>0</v>
+      </c>
+      <c r="V6" s="113">
+        <v>0</v>
+      </c>
+      <c r="W6" s="113">
+        <f>SUM(B6:V6)</f>
+        <v>0</v>
+      </c>
+      <c r="Z6"/>
     </row>
     <row r="7" spans="1:26" customHeight="1" ht="15.75">
       <c r="A7" s="116"/>
@@ -48647,6 +48705,31 @@
       <c r="V1000" s="116"/>
       <c r="W1000" s="116"/>
     </row>
+    <row r="1001" spans="1:26" customHeight="1" ht="15.75">
+      <c r="A1001" s="116"/>
+      <c r="B1001" s="116"/>
+      <c r="C1001" s="116"/>
+      <c r="D1001" s="116"/>
+      <c r="E1001" s="116"/>
+      <c r="F1001" s="116"/>
+      <c r="G1001" s="116"/>
+      <c r="H1001" s="116"/>
+      <c r="I1001" s="116"/>
+      <c r="J1001" s="116"/>
+      <c r="K1001" s="116"/>
+      <c r="L1001" s="116"/>
+      <c r="M1001" s="116"/>
+      <c r="N1001" s="116"/>
+      <c r="O1001" s="116"/>
+      <c r="P1001" s="116"/>
+      <c r="Q1001" s="116"/>
+      <c r="R1001" s="116"/>
+      <c r="S1001" s="116"/>
+      <c r="T1001" s="116"/>
+      <c r="U1001" s="116"/>
+      <c r="V1001" s="116"/>
+      <c r="W1001" s="116"/>
+    </row>
   </sheetData>
   <sheetProtection sheet="false" objects="false" scenarios="false" formatCells="false" formatColumns="false" formatRows="false" insertColumns="false" insertRows="false" insertHyperlinks="false" deleteColumns="false" deleteRows="false" selectLockedCells="false" sort="false" autoFilter="false" pivotTables="false" selectUnlockedCells="false"/>
   <mergeCells>

</xml_diff>